<commit_message>
fix new typo a5326b2ba0d566afe9958e93e8ebc298449a4654
</commit_message>
<xml_diff>
--- a/ig/nr-fix-typo/ValueSet-fr-core-practitioner-identifier-type.xlsx
+++ b/ig/nr-fix-typo/ValueSet-fr-core-practitioner-identifier-type.xlsx
@@ -38,7 +38,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>FRCoreValueSetPractitioonerIdentifierType</t>
+    <t>FRCoreValueSetPractitionerIdentifierType</t>
   </si>
   <si>
     <t>Title</t>
@@ -59,7 +59,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-06T12:59:19+00:00</t>
+    <t>2023-11-06T14:48:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>